<commit_message>
finanzas: renombrar la linea de infraestructura de La Rural
Se llamaba "Infraestructura y mobiliario de stands", lo que hacia parecer que
los US$9.270 incluian el mobiliario del publico. Pasa a llamarse
"Infraestructura La Rural (armado de stands)" y la descripcion aclara que las
sillas del publico van en su propia linea.

Sin cambios en los montos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ExCmhEkQkaZXm6WKFzKVu
</commit_message>
<xml_diff>
--- a/ops/finanzas/ARGENTINA_CMC2026_Costo_Total.xlsx
+++ b/ops/finanzas/ARGENTINA_CMC2026_Costo_Total.xlsx
@@ -1034,7 +1034,7 @@
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Infraestructura y mobiliario de stands</t>
+          <t>Infraestructura La Rural (armado de stands)</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Definido: armado de los stands y su mobiliario. Stand de staff 100 m², stand de producción menos de 50 m², y el mobiliario del camarín de speakers. Falta pedirles los espejos.</t>
+          <t>Armado del stand de staff (100 m²), el de producción (menos de 50 m²) y el mobiliario del camarín de speakers. Falta pedirles los espejos. Las sillas del público van en su propia línea.</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">

</xml_diff>

<commit_message>
finanzas: fijar el dolar en 1.510 y cerrar sillas y catering
El tipo de cambio operativo es 1.510, no 1.530. Se verifico contra dos cifras
de Agustina: el montaje de $900.000 le da US$596 y el entelado de $24.500.000
le da US$16.225. Todas las conversiones de pesos del libro se recalculan con
ese valor.

- Sillas: presupuesto FDL Eventos N.º 026-2697 del 07/08, alquiler por 4 dias.
  1.000 sillas hotel cano gris tapizado negro $7.000.000 + 4.500 plasticas
  Munro reforzadas $17.100.000 + flete $1.700.000 = $25.800.000 + IVA =
  $31.218.000 = US$20.674.
- Catering: US$14.569 (antes US$13.582).
- Montaje y desmontaje de sillas: US$596.

Costo total US$252.008 contra US$176.159 presupuestados (+43,1%).
US$42,00 por asistente pago. Ahorro negociado US$40.247 (unos $60,8 millones).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ExCmhEkQkaZXm6WKFzKVu
</commit_message>
<xml_diff>
--- a/ops/finanzas/ARGENTINA_CMC2026_Costo_Total.xlsx
+++ b/ops/finanzas/ARGENTINA_CMC2026_Costo_Total.xlsx
@@ -745,7 +745,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Celda TABLERO!C4, editable. Por defecto $1.535 = dólar oficial venta del Banco Nación al 02/09/2026. Todas las conversiones de pesos a dólares salen de esa única celda.</t>
+          <t>Celda TABLERO!C4, editable. $1.510, que es el dólar con el que viene trabajando Agustina. Se verificó contra dos de sus cifras: el montaje de $900.000 le da US$596 y el entelado de $24.500.000 le da US$16.225. Todas las conversiones de pesos a dólares salen de esa única celda.</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>4.500 sillas plásticas Munro reforzadas + 1.000 sillas hotel negro + flete. NO incluye armado.</t>
+          <t>Presupuesto 026-2697, alquiler por 4 días: 1.000 sillas hotel caño gris tapizado negro ($7.000.000) + 4.500 sillas plásticas Munro reforzadas ($17.100.000) + flete ($1.700.000). NO incluye armado.</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="L8" s="24" t="inlineStr">
         <is>
-          <t>Mail fdleventos@gmail.com 07/08/2026 · pendiente de resolver facturación al exterior</t>
+          <t>Presupuesto FDL Eventos N.º 026-2697 del 07/08/2026 · pendiente de resolver facturación al exterior</t>
         </is>
       </c>
     </row>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="F37" s="12" t="n">
-        <v>13582</v>
+        <v>14569</v>
       </c>
       <c r="G37" s="13" t="n"/>
       <c r="H37" s="14">
@@ -3073,11 +3073,11 @@
         </is>
       </c>
       <c r="C4" s="48" t="n">
-        <v>1530</v>
+        <v>1510</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Dólar oficial venta, Banco Nación, 02/09/2026. Editá esta celda y se recalcula todo el libro.</t>
+          <t>Dólar con el que trabaja Agustina. Verificado contra dos de sus cifras: $900.000 de montaje = US$596 y $24.500.000 de entelado = US$16.225. Editá esta celda y se recalcula todo el libro.</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="F8" s="19" t="n"/>
       <c r="G8" s="23" t="n">
-        <v>13582</v>
+        <v>14569</v>
       </c>
       <c r="H8" s="59">
         <f>D8-G8</f>

</xml_diff>